<commit_message>
Add Ex4A GTrends Excel file
</commit_message>
<xml_diff>
--- a/week-01/Ex4A_GTrends.xlsx
+++ b/week-01/Ex4A_GTrends.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eyerusalemdebero/Documents/DataAnalytics/week-01/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{04770F60-F90B-3840-A475-18DAA17595C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F5D72157-BB29-854D-967F-29EEF0CE23AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2140" yWindow="740" windowWidth="28040" windowHeight="17220" xr2:uid="{3A9E0413-B0AF-3F46-8F43-695D8F2641DF}"/>
   </bookViews>

</xml_diff>